<commit_message>
I have protected the sheets
</commit_message>
<xml_diff>
--- a/BookVSMovie Project.xlsx
+++ b/BookVSMovie Project.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/23955d91da42c630/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\BooksVSMovie Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2059" documentId="8_{7AAFB040-6653-4E16-A06E-B4AD1396D547}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{70558302-F46F-4D21-A99C-884F90D12D92}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45CB8E60-47F4-4AEB-974A-C7DC57246C34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="44" xr2:uid="{32A63E87-171A-461B-A186-40FC3C7CA516}"/>
   </bookViews>
@@ -1670,35 +1670,35 @@
     <xf numFmtId="0" fontId="5" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="5" fillId="8" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="3" fontId="10" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -49203,2002 +49203,1996 @@
   <dimension ref="A1:AR40"/>
   <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21" style="34" customWidth="1"/>
-    <col min="2" max="13" width="11.42578125" style="34" customWidth="1"/>
-    <col min="14" max="14" width="21" style="34" customWidth="1"/>
-    <col min="15" max="21" width="11.42578125" style="34" customWidth="1"/>
-    <col min="22" max="22" width="12.7109375" style="34"/>
-    <col min="23" max="44" width="0" style="34" hidden="1" customWidth="1"/>
-    <col min="45" max="16384" width="12.7109375" style="34"/>
+    <col min="1" max="1" width="21" style="35" customWidth="1"/>
+    <col min="2" max="13" width="11.42578125" style="35" customWidth="1"/>
+    <col min="14" max="14" width="21" style="35" customWidth="1"/>
+    <col min="15" max="21" width="11.42578125" style="35" customWidth="1"/>
+    <col min="22" max="22" width="12.7109375" style="35"/>
+    <col min="23" max="44" width="0" style="35" hidden="1" customWidth="1"/>
+    <col min="45" max="16384" width="12.7109375" style="35"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:44" ht="34.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="44" t="s">
         <v>102</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
-      <c r="I1" s="42"/>
-      <c r="J1" s="42"/>
-      <c r="K1" s="42"/>
-      <c r="L1" s="42"/>
-      <c r="M1" s="42"/>
-      <c r="N1" s="42"/>
-      <c r="O1" s="42"/>
-      <c r="P1" s="42"/>
-      <c r="Q1" s="42"/>
-      <c r="R1" s="42"/>
-      <c r="S1" s="42"/>
-      <c r="T1" s="42"/>
-      <c r="U1" s="42"/>
-      <c r="W1" s="34" t="s">
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
+      <c r="I1" s="44"/>
+      <c r="J1" s="44"/>
+      <c r="K1" s="44"/>
+      <c r="L1" s="44"/>
+      <c r="M1" s="44"/>
+      <c r="N1" s="44"/>
+      <c r="O1" s="44"/>
+      <c r="P1" s="44"/>
+      <c r="Q1" s="44"/>
+      <c r="R1" s="44"/>
+      <c r="S1" s="44"/>
+      <c r="T1" s="44"/>
+      <c r="U1" s="44"/>
+      <c r="W1" s="35" t="s">
         <v>130</v>
       </c>
-      <c r="X1" s="34" t="s">
+      <c r="X1" s="35" t="s">
         <v>131</v>
       </c>
-      <c r="Y1" s="34" t="s">
+      <c r="Y1" s="35" t="s">
         <v>132</v>
       </c>
-      <c r="AA1" s="34" t="s">
+      <c r="AA1" s="35" t="s">
         <v>130</v>
       </c>
-      <c r="AB1" s="34" t="s">
+      <c r="AB1" s="35" t="s">
         <v>161</v>
       </c>
-      <c r="AC1" s="34" t="s">
+      <c r="AC1" s="35" t="s">
         <v>162</v>
       </c>
-      <c r="AD1" s="34" t="s">
+      <c r="AD1" s="35" t="s">
         <v>163</v>
       </c>
-      <c r="AE1" s="34" t="s">
+      <c r="AE1" s="35" t="s">
         <v>164</v>
       </c>
-      <c r="AF1" s="34" t="s">
+      <c r="AF1" s="35" t="s">
         <v>165</v>
       </c>
-      <c r="AH1" s="34" t="s">
+      <c r="AH1" s="35" t="s">
         <v>130</v>
       </c>
-      <c r="AI1" s="34" t="s">
+      <c r="AI1" s="35" t="s">
         <v>166</v>
       </c>
-      <c r="AJ1" s="34" t="s">
+      <c r="AJ1" s="35" t="s">
         <v>167</v>
       </c>
-      <c r="AK1" s="34" t="s">
+      <c r="AK1" s="35" t="s">
         <v>168</v>
       </c>
-      <c r="AL1" s="34" t="s">
+      <c r="AL1" s="35" t="s">
         <v>169</v>
       </c>
-      <c r="AM1" s="34" t="s">
+      <c r="AM1" s="35" t="s">
         <v>170</v>
       </c>
-      <c r="AN1" s="34" t="s">
+      <c r="AN1" s="35" t="s">
         <v>165</v>
       </c>
-      <c r="AO1" s="34" t="s">
+      <c r="AO1" s="35" t="s">
         <v>164</v>
       </c>
-      <c r="AP1" s="34" t="s">
+      <c r="AP1" s="35" t="s">
         <v>163</v>
       </c>
-      <c r="AQ1" s="34" t="s">
+      <c r="AQ1" s="35" t="s">
         <v>162</v>
       </c>
-      <c r="AR1" s="34" t="s">
+      <c r="AR1" s="35" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="W2" s="34" t="s">
+      <c r="W2" s="35" t="s">
         <v>5</v>
       </c>
-      <c r="X2" s="34" t="s">
+      <c r="X2" s="35" t="s">
         <v>133</v>
       </c>
-      <c r="Y2" s="34" t="s">
+      <c r="Y2" s="35" t="s">
         <v>134</v>
       </c>
-      <c r="AA2" s="34" t="s">
+      <c r="AA2" s="35" t="s">
         <v>5</v>
       </c>
-      <c r="AB2" s="34">
+      <c r="AB2" s="35">
         <v>7147</v>
       </c>
-      <c r="AC2" s="34">
+      <c r="AC2" s="35">
         <v>13555</v>
       </c>
-      <c r="AD2" s="34">
+      <c r="AD2" s="35">
         <v>53778</v>
       </c>
-      <c r="AE2" s="34">
+      <c r="AE2" s="35">
         <v>160455</v>
       </c>
-      <c r="AF2" s="34">
+      <c r="AF2" s="35">
         <v>503742</v>
       </c>
-      <c r="AH2" s="34" t="s">
+      <c r="AH2" s="35" t="s">
         <v>5</v>
       </c>
-      <c r="AI2" s="34">
+      <c r="AI2" s="35">
         <v>860000</v>
       </c>
-      <c r="AJ2" s="34">
+      <c r="AJ2" s="35">
         <v>612000</v>
       </c>
-      <c r="AK2" s="34">
+      <c r="AK2" s="35">
         <v>411000</v>
       </c>
-      <c r="AL2" s="34">
+      <c r="AL2" s="35">
         <v>170000</v>
       </c>
-      <c r="AM2" s="34">
+      <c r="AM2" s="35">
         <v>59000</v>
       </c>
-      <c r="AN2" s="34">
+      <c r="AN2" s="35">
         <v>28000</v>
       </c>
-      <c r="AO2" s="34">
+      <c r="AO2" s="35">
         <v>14000</v>
       </c>
-      <c r="AP2" s="34">
+      <c r="AP2" s="35">
         <v>10000</v>
       </c>
-      <c r="AQ2" s="34">
+      <c r="AQ2" s="35">
         <v>8300</v>
       </c>
-      <c r="AR2" s="34">
+      <c r="AR2" s="35">
         <v>32000</v>
       </c>
     </row>
     <row r="3" spans="1:44" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I3" s="44" t="s">
+      <c r="I3" s="45" t="s">
         <v>103</v>
       </c>
-      <c r="J3" s="44"/>
-      <c r="K3" s="44"/>
-      <c r="L3" s="44"/>
-      <c r="M3" s="44"/>
-      <c r="W3" s="34" t="s">
+      <c r="J3" s="45"/>
+      <c r="K3" s="45"/>
+      <c r="L3" s="45"/>
+      <c r="M3" s="45"/>
+      <c r="W3" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="X3" s="34" t="s">
+      <c r="X3" s="35" t="s">
         <v>135</v>
       </c>
-      <c r="Y3" s="34" t="s">
+      <c r="Y3" s="35" t="s">
         <v>136</v>
       </c>
-      <c r="AA3" s="34" t="s">
+      <c r="AA3" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="AB3" s="34">
+      <c r="AB3" s="35">
         <v>193502</v>
       </c>
-      <c r="AC3" s="34">
+      <c r="AC3" s="35">
         <v>220459</v>
       </c>
-      <c r="AD3" s="34">
+      <c r="AD3" s="35">
         <v>988556</v>
       </c>
-      <c r="AE3" s="34">
+      <c r="AE3" s="35">
         <v>2735320</v>
       </c>
-      <c r="AF3" s="34">
+      <c r="AF3" s="35">
         <v>7440244</v>
       </c>
-      <c r="AH3" s="34" t="s">
+      <c r="AH3" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="AI3" s="34">
+      <c r="AI3" s="35">
         <v>175000</v>
       </c>
-      <c r="AJ3" s="34">
+      <c r="AJ3" s="35">
         <v>121000</v>
       </c>
-      <c r="AK3" s="34">
+      <c r="AK3" s="35">
         <v>270000</v>
       </c>
-      <c r="AL3" s="34">
+      <c r="AL3" s="35">
         <v>241000</v>
       </c>
-      <c r="AM3" s="34">
+      <c r="AM3" s="35">
         <v>87000</v>
       </c>
-      <c r="AN3" s="34">
+      <c r="AN3" s="35">
         <v>29000</v>
       </c>
-      <c r="AO3" s="34">
+      <c r="AO3" s="35">
         <v>10000</v>
       </c>
-      <c r="AP3" s="34">
+      <c r="AP3" s="35">
         <v>5300</v>
       </c>
-      <c r="AQ3" s="34">
+      <c r="AQ3" s="35">
         <v>3200</v>
       </c>
-      <c r="AR3" s="34">
+      <c r="AR3" s="35">
         <v>9300</v>
       </c>
     </row>
     <row r="4" spans="1:44" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="I4" s="43" t="s">
+      <c r="I4" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="J4" s="43"/>
-      <c r="K4" s="43"/>
-      <c r="L4" s="43"/>
-      <c r="M4" s="43"/>
-      <c r="N4" s="35"/>
-      <c r="W4" s="34" t="s">
+      <c r="J4" s="34"/>
+      <c r="K4" s="34"/>
+      <c r="L4" s="34"/>
+      <c r="M4" s="34"/>
+      <c r="N4" s="43"/>
+      <c r="W4" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="X4" s="34" t="s">
+      <c r="X4" s="35" t="s">
         <v>137</v>
       </c>
-      <c r="Y4" s="34" t="s">
+      <c r="Y4" s="35" t="s">
         <v>138</v>
       </c>
-      <c r="AA4" s="34" t="s">
+      <c r="AA4" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="AB4" s="34">
+      <c r="AB4" s="35">
         <v>27777</v>
       </c>
-      <c r="AC4" s="34">
+      <c r="AC4" s="35">
         <v>44105</v>
       </c>
-      <c r="AD4" s="34">
+      <c r="AD4" s="35">
         <v>151665</v>
       </c>
-      <c r="AE4" s="34">
+      <c r="AE4" s="35">
         <v>319713</v>
       </c>
-      <c r="AF4" s="34">
+      <c r="AF4" s="35">
         <v>719870</v>
       </c>
-      <c r="AH4" s="34" t="s">
+      <c r="AH4" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="AI4" s="34">
+      <c r="AI4" s="35">
         <v>98000</v>
       </c>
-      <c r="AJ4" s="34">
+      <c r="AJ4" s="35">
         <v>70000</v>
       </c>
-      <c r="AK4" s="34">
+      <c r="AK4" s="35">
         <v>86000</v>
       </c>
-      <c r="AL4" s="34">
+      <c r="AL4" s="35">
         <v>50000</v>
       </c>
-      <c r="AM4" s="34">
+      <c r="AM4" s="35">
         <v>23000</v>
       </c>
-      <c r="AN4" s="34">
+      <c r="AN4" s="35">
         <v>11000</v>
       </c>
-      <c r="AO4" s="34">
+      <c r="AO4" s="35">
         <v>5700</v>
       </c>
-      <c r="AP4" s="34">
+      <c r="AP4" s="35">
         <v>3800</v>
       </c>
-      <c r="AQ4" s="34">
+      <c r="AQ4" s="35">
         <v>2800</v>
       </c>
-      <c r="AR4" s="34">
+      <c r="AR4" s="35">
         <v>6200</v>
       </c>
     </row>
     <row r="5" spans="1:44" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="W5" s="34" t="s">
+      <c r="W5" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="X5" s="34" t="s">
+      <c r="X5" s="35" t="s">
         <v>139</v>
       </c>
-      <c r="Y5" s="34" t="s">
+      <c r="Y5" s="35" t="s">
         <v>140</v>
       </c>
-      <c r="AA5" s="34" t="s">
+      <c r="AA5" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="AB5" s="34">
+      <c r="AB5" s="35">
         <v>132601</v>
       </c>
-      <c r="AC5" s="34">
+      <c r="AC5" s="35">
         <v>240340</v>
       </c>
-      <c r="AD5" s="34">
+      <c r="AD5" s="35">
         <v>1104482</v>
       </c>
-      <c r="AE5" s="34">
+      <c r="AE5" s="35">
         <v>3054271</v>
       </c>
-      <c r="AF5" s="34">
+      <c r="AF5" s="35">
         <v>5534811</v>
       </c>
-      <c r="AH5" s="34" t="s">
+      <c r="AH5" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="AI5" s="34">
+      <c r="AI5" s="35">
         <v>136000</v>
       </c>
-      <c r="AJ5" s="34">
+      <c r="AJ5" s="35">
         <v>125000</v>
       </c>
-      <c r="AK5" s="34">
+      <c r="AK5" s="35">
         <v>280000</v>
       </c>
-      <c r="AL5" s="34">
+      <c r="AL5" s="35">
         <v>303000</v>
       </c>
-      <c r="AM5" s="34">
+      <c r="AM5" s="35">
         <v>131000</v>
       </c>
-      <c r="AN5" s="34">
+      <c r="AN5" s="35">
         <v>51000</v>
       </c>
-      <c r="AO5" s="34">
+      <c r="AO5" s="35">
         <v>21000</v>
       </c>
-      <c r="AP5" s="34">
+      <c r="AP5" s="35">
         <v>11000</v>
       </c>
-      <c r="AQ5" s="34">
+      <c r="AQ5" s="35">
         <v>7000</v>
       </c>
-      <c r="AR5" s="34">
+      <c r="AR5" s="35">
         <v>15000</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="W6" s="34" t="s">
+      <c r="W6" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="X6" s="34" t="s">
+      <c r="X6" s="35" t="s">
         <v>141</v>
       </c>
-      <c r="Y6" s="34" t="s">
+      <c r="Y6" s="35" t="s">
         <v>142</v>
       </c>
-      <c r="AA6" s="34" t="s">
+      <c r="AA6" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="AB6" s="34">
+      <c r="AB6" s="35">
         <v>271164</v>
       </c>
-      <c r="AC6" s="34">
+      <c r="AC6" s="35">
         <v>137019</v>
       </c>
-      <c r="AD6" s="34">
+      <c r="AD6" s="35">
         <v>46266</v>
       </c>
-      <c r="AE6" s="34">
+      <c r="AE6" s="35">
         <v>10170</v>
       </c>
-      <c r="AF6" s="34">
+      <c r="AF6" s="35">
         <v>5601</v>
       </c>
-      <c r="AH6" s="34" t="s">
+      <c r="AH6" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="AI6" s="34">
+      <c r="AI6" s="35">
         <v>1100000</v>
       </c>
-      <c r="AJ6" s="34">
+      <c r="AJ6" s="35">
         <v>557000</v>
       </c>
-      <c r="AK6" s="34">
+      <c r="AK6" s="35">
         <v>280000</v>
       </c>
-      <c r="AL6" s="34">
+      <c r="AL6" s="35">
         <v>110000</v>
       </c>
-      <c r="AM6" s="34">
+      <c r="AM6" s="35">
         <v>41000</v>
       </c>
-      <c r="AN6" s="34">
+      <c r="AN6" s="35">
         <v>22000</v>
       </c>
-      <c r="AO6" s="34">
+      <c r="AO6" s="35">
         <v>11000</v>
       </c>
-      <c r="AP6" s="34">
+      <c r="AP6" s="35">
         <v>8400</v>
       </c>
-      <c r="AQ6" s="34">
+      <c r="AQ6" s="35">
         <v>7500</v>
       </c>
-      <c r="AR6" s="34">
+      <c r="AR6" s="35">
         <v>44000</v>
       </c>
     </row>
     <row r="7" spans="1:44" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A7" s="45" t="s">
+      <c r="A7" s="36" t="s">
         <v>104</v>
       </c>
-      <c r="B7" s="45"/>
-      <c r="C7" s="45"/>
-      <c r="D7" s="45"/>
-      <c r="E7" s="45"/>
-      <c r="F7" s="45"/>
-      <c r="G7" s="45"/>
-      <c r="H7" s="45"/>
-      <c r="N7" s="45" t="s">
+      <c r="B7" s="36"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="36"/>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36"/>
+      <c r="G7" s="36"/>
+      <c r="H7" s="36"/>
+      <c r="N7" s="36" t="s">
         <v>105</v>
       </c>
-      <c r="O7" s="45"/>
-      <c r="P7" s="45"/>
-      <c r="Q7" s="45"/>
-      <c r="R7" s="45"/>
-      <c r="S7" s="45"/>
-      <c r="T7" s="45"/>
-      <c r="U7" s="45"/>
-      <c r="W7" s="34" t="s">
+      <c r="O7" s="36"/>
+      <c r="P7" s="36"/>
+      <c r="Q7" s="36"/>
+      <c r="R7" s="36"/>
+      <c r="S7" s="36"/>
+      <c r="T7" s="36"/>
+      <c r="U7" s="36"/>
+      <c r="W7" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="X7" s="34" t="s">
+      <c r="X7" s="35" t="s">
         <v>143</v>
       </c>
-      <c r="Y7" s="34" t="s">
+      <c r="Y7" s="35" t="s">
         <v>144</v>
       </c>
-      <c r="AA7" s="34" t="s">
+      <c r="AA7" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="AB7" s="34">
+      <c r="AB7" s="35">
         <v>3597983</v>
       </c>
-      <c r="AC7" s="34">
+      <c r="AC7" s="35">
         <v>2092922</v>
       </c>
-      <c r="AD7" s="34">
+      <c r="AD7" s="35">
         <v>925028</v>
       </c>
-      <c r="AE7" s="34">
+      <c r="AE7" s="35">
         <v>241851</v>
       </c>
-      <c r="AF7" s="34">
+      <c r="AF7" s="35">
         <v>126635</v>
       </c>
-      <c r="AH7" s="34" t="s">
+      <c r="AH7" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="AI7" s="34">
+      <c r="AI7" s="35">
         <v>77000</v>
       </c>
-      <c r="AJ7" s="34">
+      <c r="AJ7" s="35">
         <v>84000</v>
       </c>
-      <c r="AK7" s="34">
+      <c r="AK7" s="35">
         <v>101000</v>
       </c>
-      <c r="AL7" s="34">
+      <c r="AL7" s="35">
         <v>53000</v>
       </c>
-      <c r="AM7" s="34">
+      <c r="AM7" s="35">
         <v>19000</v>
       </c>
-      <c r="AN7" s="34">
+      <c r="AN7" s="35">
         <v>7900</v>
       </c>
-      <c r="AO7" s="34">
+      <c r="AO7" s="35">
         <v>3400</v>
       </c>
-      <c r="AP7" s="34">
+      <c r="AP7" s="35">
         <v>1900</v>
       </c>
-      <c r="AQ7" s="34">
+      <c r="AQ7" s="35">
         <v>1400</v>
       </c>
-      <c r="AR7" s="34">
+      <c r="AR7" s="35">
         <v>4200</v>
       </c>
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="W8" s="34" t="s">
+      <c r="W8" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="X8" s="34" t="s">
+      <c r="X8" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="Y8" s="34" t="s">
+      <c r="Y8" s="35" t="s">
         <v>145</v>
       </c>
-      <c r="AA8" s="34" t="s">
+      <c r="AA8" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="AB8" s="34">
+      <c r="AB8" s="35">
         <v>2700215</v>
       </c>
-      <c r="AC8" s="34">
+      <c r="AC8" s="35">
         <v>1331924</v>
       </c>
-      <c r="AD8" s="34">
+      <c r="AD8" s="35">
         <v>580632</v>
       </c>
-      <c r="AE8" s="34">
+      <c r="AE8" s="35">
         <v>169365</v>
       </c>
-      <c r="AF8" s="34">
+      <c r="AF8" s="35">
         <v>111189</v>
       </c>
-      <c r="AH8" s="34" t="s">
+      <c r="AH8" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="AI8" s="34">
+      <c r="AI8" s="35">
         <v>85000</v>
       </c>
-      <c r="AJ8" s="34">
+      <c r="AJ8" s="35">
         <v>62000</v>
       </c>
-      <c r="AK8" s="34">
+      <c r="AK8" s="35">
         <v>102000</v>
       </c>
-      <c r="AL8" s="34">
+      <c r="AL8" s="35">
         <v>74000</v>
       </c>
-      <c r="AM8" s="34">
+      <c r="AM8" s="35">
         <v>29000</v>
       </c>
-      <c r="AN8" s="34">
+      <c r="AN8" s="35">
         <v>11000</v>
       </c>
-      <c r="AO8" s="34">
+      <c r="AO8" s="35">
         <v>4600</v>
       </c>
-      <c r="AP8" s="34">
+      <c r="AP8" s="35">
         <v>2600</v>
       </c>
-      <c r="AQ8" s="34">
+      <c r="AQ8" s="35">
         <v>1800</v>
       </c>
-      <c r="AR8" s="34">
+      <c r="AR8" s="35">
         <v>3700</v>
       </c>
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A9" s="36" t="s">
+      <c r="A9" s="37" t="s">
         <v>120</v>
       </c>
-      <c r="B9" s="40" t="str">
+      <c r="B9" s="38" t="str">
         <f>INDEX(Table2[Book Title],MATCH(I4,Table2[Book Title],0))</f>
         <v>The Godfather (The Godfather, #1)</v>
       </c>
-      <c r="C9" s="40"/>
-      <c r="D9" s="40"/>
-      <c r="E9" s="40"/>
-      <c r="F9" s="40"/>
-      <c r="G9" s="40"/>
-      <c r="H9" s="40"/>
-      <c r="N9" s="36" t="s">
+      <c r="C9" s="38"/>
+      <c r="D9" s="38"/>
+      <c r="E9" s="38"/>
+      <c r="F9" s="38"/>
+      <c r="G9" s="38"/>
+      <c r="H9" s="38"/>
+      <c r="N9" s="37" t="s">
         <v>119</v>
       </c>
-      <c r="O9" s="40" t="str">
+      <c r="O9" s="38" t="str">
         <f>INDEX('Movie Data'!C2:C21,MATCH(I4,Table2[Book Title],0))</f>
         <v>The Godfather</v>
       </c>
-      <c r="P9" s="40"/>
-      <c r="Q9" s="40"/>
-      <c r="R9" s="40"/>
-      <c r="S9" s="40"/>
-      <c r="T9" s="40"/>
-      <c r="U9" s="40"/>
-      <c r="W9" s="34" t="s">
+      <c r="P9" s="38"/>
+      <c r="Q9" s="38"/>
+      <c r="R9" s="38"/>
+      <c r="S9" s="38"/>
+      <c r="T9" s="38"/>
+      <c r="U9" s="38"/>
+      <c r="W9" s="35" t="s">
         <v>44</v>
       </c>
-      <c r="X9" s="34" t="s">
+      <c r="X9" s="35" t="s">
         <v>58</v>
       </c>
-      <c r="Y9" s="34" t="s">
+      <c r="Y9" s="35" t="s">
         <v>146</v>
       </c>
-      <c r="AA9" s="34" t="s">
+      <c r="AA9" s="35" t="s">
         <v>44</v>
       </c>
-      <c r="AB9" s="34">
+      <c r="AB9" s="35">
         <v>295546</v>
       </c>
-      <c r="AC9" s="34">
+      <c r="AC9" s="35">
         <v>196000</v>
       </c>
-      <c r="AD9" s="34">
+      <c r="AD9" s="35">
         <v>74186</v>
       </c>
-      <c r="AE9" s="34">
+      <c r="AE9" s="35">
         <v>16097</v>
       </c>
-      <c r="AF9" s="34">
+      <c r="AF9" s="35">
         <v>11741</v>
       </c>
-      <c r="AH9" s="34" t="s">
+      <c r="AH9" s="35" t="s">
         <v>44</v>
       </c>
-      <c r="AI9" s="34">
+      <c r="AI9" s="35">
         <v>407000</v>
       </c>
-      <c r="AJ9" s="34">
+      <c r="AJ9" s="35">
         <v>563000</v>
       </c>
-      <c r="AK9" s="34">
+      <c r="AK9" s="35">
         <v>482000</v>
       </c>
-      <c r="AL9" s="34">
+      <c r="AL9" s="35">
         <v>182000</v>
       </c>
-      <c r="AM9" s="34">
+      <c r="AM9" s="35">
         <v>48000</v>
       </c>
-      <c r="AN9" s="34">
+      <c r="AN9" s="35">
         <v>17000</v>
       </c>
-      <c r="AO9" s="34">
+      <c r="AO9" s="35">
         <v>7400</v>
       </c>
-      <c r="AP9" s="34">
+      <c r="AP9" s="35">
         <v>4200</v>
       </c>
-      <c r="AQ9" s="34">
+      <c r="AQ9" s="35">
         <v>3200</v>
       </c>
-      <c r="AR9" s="34">
+      <c r="AR9" s="35">
         <v>7600</v>
       </c>
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A10" s="36" t="s">
+      <c r="A10" s="37" t="s">
         <v>121</v>
       </c>
-      <c r="B10" s="40" t="str">
+      <c r="B10" s="38" t="str">
         <f>INDEX(Table2[Author],MATCH(I4,Table2[Book Title],0))</f>
         <v>Mario Puzo</v>
       </c>
-      <c r="C10" s="40"/>
-      <c r="D10" s="40"/>
-      <c r="E10" s="40"/>
-      <c r="F10" s="40"/>
-      <c r="G10" s="40"/>
-      <c r="H10" s="40"/>
-      <c r="N10" s="36" t="s">
+      <c r="C10" s="38"/>
+      <c r="D10" s="38"/>
+      <c r="E10" s="38"/>
+      <c r="F10" s="38"/>
+      <c r="G10" s="38"/>
+      <c r="H10" s="38"/>
+      <c r="N10" s="37" t="s">
         <v>123</v>
       </c>
-      <c r="O10" s="40" t="str">
+      <c r="O10" s="38" t="str">
         <f>INDEX('Movie Data'!$D$2:$D$21,MATCH(I4,Table2[Book Title],0))</f>
         <v>Francis Ford Coppola</v>
       </c>
-      <c r="P10" s="40"/>
-      <c r="Q10" s="40"/>
-      <c r="R10" s="40"/>
-      <c r="S10" s="40"/>
-      <c r="T10" s="40"/>
-      <c r="U10" s="40"/>
-      <c r="W10" s="34" t="s">
+      <c r="P10" s="38"/>
+      <c r="Q10" s="38"/>
+      <c r="R10" s="38"/>
+      <c r="S10" s="38"/>
+      <c r="T10" s="38"/>
+      <c r="U10" s="38"/>
+      <c r="W10" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="X10" s="34" t="s">
+      <c r="X10" s="35" t="s">
         <v>147</v>
       </c>
-      <c r="Y10" s="34" t="s">
+      <c r="Y10" s="35" t="s">
         <v>148</v>
       </c>
-      <c r="AA10" s="34" t="s">
+      <c r="AA10" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="AB10" s="34">
+      <c r="AB10" s="35">
         <v>1632451</v>
       </c>
-      <c r="AC10" s="34">
+      <c r="AC10" s="35">
         <v>1152649</v>
       </c>
-      <c r="AD10" s="34">
+      <c r="AD10" s="35">
         <v>469607</v>
       </c>
-      <c r="AE10" s="34">
+      <c r="AE10" s="35">
         <v>134311</v>
       </c>
-      <c r="AF10" s="34">
+      <c r="AF10" s="35">
         <v>93029</v>
       </c>
-      <c r="AH10" s="34" t="s">
+      <c r="AH10" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="AI10" s="34">
+      <c r="AI10" s="35">
         <v>56000</v>
       </c>
-      <c r="AJ10" s="34">
+      <c r="AJ10" s="35">
         <v>98000</v>
       </c>
-      <c r="AK10" s="34">
+      <c r="AK10" s="35">
         <v>192000</v>
       </c>
-      <c r="AL10" s="34">
+      <c r="AL10" s="35">
         <v>118000</v>
       </c>
-      <c r="AM10" s="34">
+      <c r="AM10" s="35">
         <v>37000</v>
       </c>
-      <c r="AN10" s="34">
+      <c r="AN10" s="35">
         <v>12000</v>
       </c>
-      <c r="AO10" s="34">
+      <c r="AO10" s="35">
         <v>4900</v>
       </c>
-      <c r="AP10" s="34">
+      <c r="AP10" s="35">
         <v>2600</v>
       </c>
-      <c r="AQ10" s="34">
+      <c r="AQ10" s="35">
         <v>1800</v>
       </c>
-      <c r="AR10" s="34">
+      <c r="AR10" s="35">
         <v>4400</v>
       </c>
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A11" s="36" t="s">
+      <c r="A11" s="37" t="s">
         <v>124</v>
       </c>
-      <c r="B11" s="40" t="str">
+      <c r="B11" s="38" t="str">
         <f>INDEX('Books Dataset'!$G$2:$G$21,MATCH(I4,Table2[Book Title],0))</f>
         <v>Crime Fiction</v>
       </c>
-      <c r="C11" s="40"/>
-      <c r="D11" s="40"/>
-      <c r="E11" s="40"/>
-      <c r="F11" s="40"/>
-      <c r="G11" s="40"/>
-      <c r="H11" s="40"/>
-      <c r="N11" s="36" t="s">
+      <c r="C11" s="38"/>
+      <c r="D11" s="38"/>
+      <c r="E11" s="38"/>
+      <c r="F11" s="38"/>
+      <c r="G11" s="38"/>
+      <c r="H11" s="38"/>
+      <c r="N11" s="37" t="s">
         <v>124</v>
       </c>
-      <c r="O11" s="40" t="str">
+      <c r="O11" s="38" t="str">
         <f>INDEX('Books Dataset'!$G$2:$G$21,MATCH(I4,Table2[Book Title],0))</f>
         <v>Crime Fiction</v>
       </c>
-      <c r="P11" s="40"/>
-      <c r="Q11" s="40"/>
-      <c r="R11" s="40"/>
-      <c r="S11" s="40"/>
-      <c r="T11" s="40"/>
-      <c r="U11" s="40"/>
-      <c r="W11" s="34" t="s">
+      <c r="P11" s="38"/>
+      <c r="Q11" s="38"/>
+      <c r="R11" s="38"/>
+      <c r="S11" s="38"/>
+      <c r="T11" s="38"/>
+      <c r="U11" s="38"/>
+      <c r="W11" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="X11" s="34" t="s">
+      <c r="X11" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="Y11" s="34" t="s">
+      <c r="Y11" s="35" t="s">
         <v>149</v>
       </c>
-      <c r="AA11" s="34" t="s">
+      <c r="AA11" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="AB11" s="34">
+      <c r="AB11" s="35">
         <v>1703351</v>
       </c>
-      <c r="AC11" s="34">
+      <c r="AC11" s="35">
         <v>747409</v>
       </c>
-      <c r="AD11" s="34">
+      <c r="AD11" s="35">
         <v>216194</v>
       </c>
-      <c r="AE11" s="34">
+      <c r="AE11" s="35">
         <v>57020</v>
       </c>
-      <c r="AF11" s="34">
+      <c r="AF11" s="35">
         <v>44703</v>
       </c>
-      <c r="AH11" s="34" t="s">
+      <c r="AH11" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="AI11" s="34">
+      <c r="AI11" s="35">
         <v>1500000</v>
       </c>
-      <c r="AJ11" s="34">
+      <c r="AJ11" s="35">
         <v>600000</v>
       </c>
-      <c r="AK11" s="34">
+      <c r="AK11" s="35">
         <v>259000</v>
       </c>
-      <c r="AL11" s="34">
+      <c r="AL11" s="35">
         <v>99000</v>
       </c>
-      <c r="AM11" s="34">
+      <c r="AM11" s="35">
         <v>38000</v>
       </c>
-      <c r="AN11" s="34">
+      <c r="AN11" s="35">
         <v>22000</v>
       </c>
-      <c r="AO11" s="34">
+      <c r="AO11" s="35">
         <v>11000</v>
       </c>
-      <c r="AP11" s="34">
+      <c r="AP11" s="35">
         <v>9700</v>
       </c>
-      <c r="AQ11" s="34">
+      <c r="AQ11" s="35">
         <v>11000</v>
       </c>
-      <c r="AR11" s="34">
+      <c r="AR11" s="35">
         <v>85000</v>
       </c>
     </row>
     <row r="12" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A12" s="36" t="s">
+      <c r="A12" s="37" t="s">
         <v>122</v>
       </c>
-      <c r="B12" s="40">
+      <c r="B12" s="38">
         <f>INDEX(Table2[Average Rating],MATCH(I4,Table2[Book Title],0))</f>
         <v>4.4000000000000004</v>
       </c>
-      <c r="C12" s="40"/>
-      <c r="D12" s="40"/>
-      <c r="E12" s="40"/>
-      <c r="F12" s="40"/>
-      <c r="G12" s="40"/>
-      <c r="H12" s="40"/>
-      <c r="N12" s="36" t="s">
+      <c r="C12" s="38"/>
+      <c r="D12" s="38"/>
+      <c r="E12" s="38"/>
+      <c r="F12" s="38"/>
+      <c r="G12" s="38"/>
+      <c r="H12" s="38"/>
+      <c r="N12" s="37" t="s">
         <v>125</v>
       </c>
-      <c r="O12" s="40">
+      <c r="O12" s="38">
         <f>INDEX('Movie Data'!$F$2:$F$21,MATCH(I4,Table2[Book Title],0))</f>
         <v>9.1999999999999993</v>
       </c>
-      <c r="P12" s="40"/>
-      <c r="Q12" s="40"/>
-      <c r="R12" s="40"/>
-      <c r="S12" s="40"/>
-      <c r="T12" s="40"/>
-      <c r="U12" s="40"/>
-      <c r="W12" s="34" t="s">
+      <c r="P12" s="38"/>
+      <c r="Q12" s="38"/>
+      <c r="R12" s="38"/>
+      <c r="S12" s="38"/>
+      <c r="T12" s="38"/>
+      <c r="U12" s="38"/>
+      <c r="W12" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="X12" s="34" t="s">
+      <c r="X12" s="35" t="s">
         <v>57</v>
       </c>
-      <c r="Y12" s="34" t="s">
+      <c r="Y12" s="35" t="s">
         <v>150</v>
       </c>
-      <c r="AA12" s="34" t="s">
+      <c r="AA12" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="AB12" s="34">
+      <c r="AB12" s="35">
         <v>886794</v>
       </c>
-      <c r="AC12" s="34">
+      <c r="AC12" s="35">
         <v>557008</v>
       </c>
-      <c r="AD12" s="34">
+      <c r="AD12" s="35">
         <v>213163</v>
       </c>
-      <c r="AE12" s="34">
+      <c r="AE12" s="35">
         <v>47603</v>
       </c>
-      <c r="AF12" s="34">
+      <c r="AF12" s="35">
         <v>28869</v>
       </c>
-      <c r="AH12" s="34" t="s">
+      <c r="AH12" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="AI12" s="34">
+      <c r="AI12" s="35">
         <v>274000</v>
       </c>
-      <c r="AJ12" s="34">
+      <c r="AJ12" s="35">
         <v>332000</v>
       </c>
-      <c r="AK12" s="34">
+      <c r="AK12" s="35">
         <v>339000</v>
       </c>
-      <c r="AL12" s="34">
+      <c r="AL12" s="35">
         <v>165000</v>
       </c>
-      <c r="AM12" s="34">
+      <c r="AM12" s="35">
         <v>59000</v>
       </c>
-      <c r="AN12" s="34">
+      <c r="AN12" s="35">
         <v>24000</v>
       </c>
-      <c r="AO12" s="34">
+      <c r="AO12" s="35">
         <v>11000</v>
       </c>
-      <c r="AP12" s="34">
+      <c r="AP12" s="35">
         <v>6600</v>
       </c>
-      <c r="AQ12" s="34">
+      <c r="AQ12" s="35">
         <v>4500</v>
       </c>
-      <c r="AR12" s="34">
+      <c r="AR12" s="35">
         <v>8900</v>
       </c>
     </row>
     <row r="13" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A13" s="36" t="s">
+      <c r="A13" s="37" t="s">
         <v>126</v>
       </c>
-      <c r="B13" s="38">
+      <c r="B13" s="39">
         <f>INDEX(Table2[Rating Number],MATCH(I4,Table2[Book Title],0))</f>
         <v>469814</v>
       </c>
-      <c r="C13" s="38"/>
-      <c r="D13" s="38"/>
-      <c r="E13" s="38"/>
-      <c r="F13" s="38"/>
-      <c r="G13" s="38"/>
-      <c r="H13" s="38"/>
-      <c r="N13" s="36" t="s">
+      <c r="C13" s="39"/>
+      <c r="D13" s="39"/>
+      <c r="E13" s="39"/>
+      <c r="F13" s="39"/>
+      <c r="G13" s="39"/>
+      <c r="H13" s="39"/>
+      <c r="N13" s="37" t="s">
         <v>127</v>
       </c>
-      <c r="O13" s="38">
+      <c r="O13" s="39">
         <f>INDEX('Movie Data'!$G$2:$G$21,MATCH(I4,Table2[Book Title],0))*1000000</f>
         <v>2100000</v>
       </c>
-      <c r="P13" s="41"/>
-      <c r="Q13" s="41"/>
-      <c r="R13" s="41"/>
-      <c r="S13" s="41"/>
-      <c r="T13" s="41"/>
-      <c r="U13" s="41"/>
-      <c r="W13" s="34" t="s">
+      <c r="P13" s="40"/>
+      <c r="Q13" s="40"/>
+      <c r="R13" s="40"/>
+      <c r="S13" s="40"/>
+      <c r="T13" s="40"/>
+      <c r="U13" s="40"/>
+      <c r="W13" s="35" t="s">
         <v>24</v>
       </c>
-      <c r="X13" s="34" t="s">
+      <c r="X13" s="35" t="s">
         <v>52</v>
       </c>
-      <c r="Y13" s="34" t="s">
+      <c r="Y13" s="35" t="s">
         <v>151</v>
       </c>
-      <c r="AA13" s="34" t="s">
+      <c r="AA13" s="35" t="s">
         <v>24</v>
       </c>
-      <c r="AB13" s="34">
+      <c r="AB13" s="35">
         <v>927932</v>
       </c>
-      <c r="AC13" s="34">
+      <c r="AC13" s="35">
         <v>506232</v>
       </c>
-      <c r="AD13" s="34">
+      <c r="AD13" s="35">
         <v>275426</v>
       </c>
-      <c r="AE13" s="34">
+      <c r="AE13" s="35">
         <v>90333</v>
       </c>
-      <c r="AF13" s="34">
+      <c r="AF13" s="35">
         <v>55090</v>
       </c>
-      <c r="AH13" s="34" t="s">
+      <c r="AH13" s="35" t="s">
         <v>24</v>
       </c>
-      <c r="AI13" s="34">
+      <c r="AI13" s="35">
         <v>157000</v>
       </c>
-      <c r="AJ13" s="34">
+      <c r="AJ13" s="35">
         <v>122000</v>
       </c>
-      <c r="AK13" s="34">
+      <c r="AK13" s="35">
         <v>184000</v>
       </c>
-      <c r="AL13" s="34">
+      <c r="AL13" s="35">
         <v>122000</v>
       </c>
-      <c r="AM13" s="34">
+      <c r="AM13" s="35">
         <v>53000</v>
       </c>
-      <c r="AN13" s="34">
+      <c r="AN13" s="35">
         <v>23000</v>
       </c>
-      <c r="AO13" s="34">
+      <c r="AO13" s="35">
         <v>10000</v>
       </c>
-      <c r="AP13" s="34">
+      <c r="AP13" s="35">
         <v>5700</v>
       </c>
-      <c r="AQ13" s="34">
+      <c r="AQ13" s="35">
         <v>3900</v>
       </c>
-      <c r="AR13" s="34">
+      <c r="AR13" s="35">
         <v>8000</v>
       </c>
     </row>
     <row r="14" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A14" s="36" t="s">
+      <c r="A14" s="37" t="s">
         <v>128</v>
       </c>
-      <c r="B14" s="38">
+      <c r="B14" s="39">
         <f>INDEX(Table2[Copies Sold (millions)],MATCH(I4,Table2[Book Title],0))</f>
         <v>21</v>
       </c>
-      <c r="C14" s="38"/>
-      <c r="D14" s="38"/>
-      <c r="E14" s="38"/>
-      <c r="F14" s="38"/>
-      <c r="G14" s="38"/>
-      <c r="H14" s="38"/>
-      <c r="N14" s="36" t="s">
+      <c r="C14" s="39"/>
+      <c r="D14" s="39"/>
+      <c r="E14" s="39"/>
+      <c r="F14" s="39"/>
+      <c r="G14" s="39"/>
+      <c r="H14" s="39"/>
+      <c r="N14" s="37" t="s">
         <v>129</v>
       </c>
-      <c r="O14" s="38">
+      <c r="O14" s="39">
         <f>INDEX('Movie Data'!$H$2:$H$21,MATCH(I4,Table2[Book Title],0))</f>
         <v>250</v>
       </c>
-      <c r="P14" s="39"/>
-      <c r="Q14" s="39"/>
-      <c r="R14" s="39"/>
-      <c r="S14" s="39"/>
-      <c r="T14" s="39"/>
-      <c r="U14" s="39"/>
-      <c r="W14" s="34" t="s">
+      <c r="P14" s="41"/>
+      <c r="Q14" s="41"/>
+      <c r="R14" s="41"/>
+      <c r="S14" s="41"/>
+      <c r="T14" s="41"/>
+      <c r="U14" s="41"/>
+      <c r="W14" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="X14" s="34" t="s">
+      <c r="X14" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="Y14" s="34" t="s">
+      <c r="Y14" s="35" t="s">
         <v>152</v>
       </c>
-      <c r="AA14" s="34" t="s">
+      <c r="AA14" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="AB14" s="34">
+      <c r="AB14" s="35">
         <v>348155</v>
       </c>
-      <c r="AC14" s="34">
+      <c r="AC14" s="35">
         <v>288979</v>
       </c>
-      <c r="AD14" s="34">
+      <c r="AD14" s="35">
         <v>116427</v>
       </c>
-      <c r="AE14" s="34">
+      <c r="AE14" s="35">
         <v>24635</v>
       </c>
-      <c r="AF14" s="34">
+      <c r="AF14" s="35">
         <v>8754</v>
       </c>
-      <c r="AH14" s="34" t="s">
+      <c r="AH14" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="AI14" s="34">
+      <c r="AI14" s="35">
         <v>316000</v>
       </c>
-      <c r="AJ14" s="34">
+      <c r="AJ14" s="35">
         <v>368000</v>
       </c>
-      <c r="AK14" s="34">
+      <c r="AK14" s="35">
         <v>287000</v>
       </c>
-      <c r="AL14" s="34">
+      <c r="AL14" s="35">
         <v>116000</v>
       </c>
-      <c r="AM14" s="34">
+      <c r="AM14" s="35">
         <v>35000</v>
       </c>
-      <c r="AN14" s="34">
+      <c r="AN14" s="35">
         <v>13000</v>
       </c>
-      <c r="AO14" s="34">
+      <c r="AO14" s="35">
         <v>5900</v>
       </c>
-      <c r="AP14" s="34">
+      <c r="AP14" s="35">
         <v>3300</v>
       </c>
-      <c r="AQ14" s="34">
+      <c r="AQ14" s="35">
         <v>2400</v>
       </c>
-      <c r="AR14" s="34">
+      <c r="AR14" s="35">
         <v>8900</v>
       </c>
     </row>
     <row r="15" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="W15" s="34" t="s">
+      <c r="W15" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="X15" s="34" t="s">
+      <c r="X15" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="Y15" s="34" t="s">
+      <c r="Y15" s="35" t="s">
         <v>153</v>
       </c>
-      <c r="AA15" s="34" t="s">
+      <c r="AA15" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="AB15" s="34">
+      <c r="AB15" s="35">
         <v>566663</v>
       </c>
-      <c r="AC15" s="34">
+      <c r="AC15" s="35">
         <v>533792</v>
       </c>
-      <c r="AD15" s="34">
+      <c r="AD15" s="35">
         <v>305058</v>
       </c>
-      <c r="AE15" s="34">
+      <c r="AE15" s="35">
         <v>72961</v>
       </c>
-      <c r="AF15" s="34">
+      <c r="AF15" s="35">
         <v>26077</v>
       </c>
-      <c r="AH15" s="34" t="s">
+      <c r="AH15" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="AI15" s="34">
+      <c r="AI15" s="35">
         <v>34000</v>
       </c>
-      <c r="AJ15" s="34">
+      <c r="AJ15" s="35">
         <v>36000</v>
       </c>
-      <c r="AK15" s="34">
+      <c r="AK15" s="35">
         <v>73000</v>
       </c>
-      <c r="AL15" s="34">
+      <c r="AL15" s="35">
         <v>67000</v>
       </c>
-      <c r="AM15" s="34">
+      <c r="AM15" s="35">
         <v>32000</v>
       </c>
-      <c r="AN15" s="34">
+      <c r="AN15" s="35">
         <v>13000</v>
       </c>
-      <c r="AO15" s="34">
+      <c r="AO15" s="35">
         <v>6100</v>
       </c>
-      <c r="AP15" s="34">
+      <c r="AP15" s="35">
         <v>3200</v>
       </c>
-      <c r="AQ15" s="34">
+      <c r="AQ15" s="35">
         <v>2000</v>
       </c>
-      <c r="AR15" s="34">
+      <c r="AR15" s="35">
         <v>2800</v>
       </c>
     </row>
     <row r="16" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A16" s="37"/>
-      <c r="B16" s="37"/>
-      <c r="C16" s="37"/>
-      <c r="D16" s="37"/>
-      <c r="E16" s="37"/>
-      <c r="F16" s="37"/>
-      <c r="G16" s="37"/>
-      <c r="H16" s="37"/>
-      <c r="I16" s="37"/>
-      <c r="J16" s="37"/>
-      <c r="K16" s="37"/>
-      <c r="L16" s="37"/>
-      <c r="M16" s="37"/>
-      <c r="N16" s="37"/>
-      <c r="O16" s="37"/>
-      <c r="P16" s="37"/>
-      <c r="Q16" s="37"/>
-      <c r="R16" s="37"/>
-      <c r="S16" s="37"/>
-      <c r="T16" s="37"/>
-      <c r="U16" s="37"/>
-      <c r="W16" s="34" t="s">
+      <c r="A16" s="42"/>
+      <c r="B16" s="42"/>
+      <c r="C16" s="42"/>
+      <c r="D16" s="42"/>
+      <c r="E16" s="42"/>
+      <c r="F16" s="42"/>
+      <c r="G16" s="42"/>
+      <c r="H16" s="42"/>
+      <c r="I16" s="42"/>
+      <c r="J16" s="42"/>
+      <c r="K16" s="42"/>
+      <c r="L16" s="42"/>
+      <c r="M16" s="42"/>
+      <c r="N16" s="42"/>
+      <c r="O16" s="42"/>
+      <c r="P16" s="42"/>
+      <c r="Q16" s="42"/>
+      <c r="R16" s="42"/>
+      <c r="S16" s="42"/>
+      <c r="T16" s="42"/>
+      <c r="U16" s="42"/>
+      <c r="W16" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="X16" s="34" t="s">
+      <c r="X16" s="35" t="s">
         <v>54</v>
       </c>
-      <c r="Y16" s="34" t="s">
+      <c r="Y16" s="35" t="s">
         <v>154</v>
       </c>
-      <c r="AA16" s="34" t="s">
+      <c r="AA16" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="AB16" s="34">
+      <c r="AB16" s="35">
         <v>460528</v>
       </c>
-      <c r="AC16" s="34">
+      <c r="AC16" s="35">
         <v>376689</v>
       </c>
-      <c r="AD16" s="34">
+      <c r="AD16" s="35">
         <v>180717</v>
       </c>
-      <c r="AE16" s="34">
+      <c r="AE16" s="35">
         <v>40319</v>
       </c>
-      <c r="AF16" s="34">
+      <c r="AF16" s="35">
         <v>17971</v>
       </c>
-      <c r="AH16" s="34" t="s">
+      <c r="AH16" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="AI16" s="34">
+      <c r="AI16" s="35">
         <v>226000</v>
       </c>
-      <c r="AJ16" s="34">
+      <c r="AJ16" s="35">
         <v>253000</v>
       </c>
-      <c r="AK16" s="34">
+      <c r="AK16" s="35">
         <v>384000</v>
       </c>
-      <c r="AL16" s="34">
+      <c r="AL16" s="35">
         <v>204000</v>
       </c>
-      <c r="AM16" s="34">
+      <c r="AM16" s="35">
         <v>65000</v>
       </c>
-      <c r="AN16" s="34">
+      <c r="AN16" s="35">
         <v>23000</v>
       </c>
-      <c r="AO16" s="34">
+      <c r="AO16" s="35">
         <v>9100</v>
       </c>
-      <c r="AP16" s="34">
+      <c r="AP16" s="35">
         <v>5000</v>
       </c>
-      <c r="AQ16" s="34">
+      <c r="AQ16" s="35">
         <v>3000</v>
       </c>
-      <c r="AR16" s="34">
+      <c r="AR16" s="35">
         <v>5500</v>
       </c>
     </row>
     <row r="17" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A17" s="37"/>
-      <c r="B17" s="37"/>
-      <c r="C17" s="37"/>
-      <c r="D17" s="37"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="37"/>
-      <c r="G17" s="37"/>
-      <c r="H17" s="37"/>
-      <c r="I17" s="37"/>
-      <c r="J17" s="37"/>
-      <c r="K17" s="37"/>
-      <c r="L17" s="37"/>
-      <c r="M17" s="37"/>
-      <c r="N17" s="37"/>
-      <c r="O17" s="37"/>
-      <c r="P17" s="37"/>
-      <c r="Q17" s="37"/>
-      <c r="R17" s="37"/>
-      <c r="S17" s="37"/>
-      <c r="T17" s="37"/>
-      <c r="U17" s="37"/>
-      <c r="W17" s="34" t="s">
+      <c r="A17" s="42"/>
+      <c r="B17" s="42"/>
+      <c r="C17" s="42"/>
+      <c r="D17" s="42"/>
+      <c r="E17" s="42"/>
+      <c r="F17" s="42"/>
+      <c r="G17" s="42"/>
+      <c r="H17" s="42"/>
+      <c r="I17" s="42"/>
+      <c r="J17" s="42"/>
+      <c r="K17" s="42"/>
+      <c r="L17" s="42"/>
+      <c r="M17" s="42"/>
+      <c r="N17" s="42"/>
+      <c r="O17" s="42"/>
+      <c r="P17" s="42"/>
+      <c r="Q17" s="42"/>
+      <c r="R17" s="42"/>
+      <c r="S17" s="42"/>
+      <c r="T17" s="42"/>
+      <c r="U17" s="42"/>
+      <c r="W17" s="35" t="s">
         <v>31</v>
       </c>
-      <c r="X17" s="34" t="s">
+      <c r="X17" s="35" t="s">
         <v>31</v>
       </c>
-      <c r="Y17" s="34" t="s">
+      <c r="Y17" s="35" t="s">
         <v>155</v>
       </c>
-      <c r="AA17" s="34" t="s">
+      <c r="AA17" s="35" t="s">
         <v>31</v>
       </c>
-      <c r="AB17" s="34">
+      <c r="AB17" s="35">
         <v>2112564</v>
       </c>
-      <c r="AC17" s="34">
+      <c r="AC17" s="35">
         <v>2049922</v>
       </c>
-      <c r="AD17" s="34">
+      <c r="AD17" s="35">
         <v>1301238</v>
       </c>
-      <c r="AE17" s="34">
+      <c r="AE17" s="35">
         <v>383743</v>
       </c>
-      <c r="AF17" s="34">
+      <c r="AF17" s="35">
         <v>163293</v>
       </c>
-      <c r="AH17" s="34" t="s">
+      <c r="AH17" s="35" t="s">
         <v>31</v>
       </c>
-      <c r="AI17" s="34">
+      <c r="AI17" s="35">
         <v>67000</v>
       </c>
-      <c r="AJ17" s="34">
+      <c r="AJ17" s="35">
         <v>75000</v>
       </c>
-      <c r="AK17" s="34">
+      <c r="AK17" s="35">
         <v>165000</v>
       </c>
-      <c r="AL17" s="34">
+      <c r="AL17" s="35">
         <v>182000</v>
       </c>
-      <c r="AM17" s="34">
+      <c r="AM17" s="35">
         <v>89000</v>
       </c>
-      <c r="AN17" s="34">
+      <c r="AN17" s="35">
         <v>35000</v>
       </c>
-      <c r="AO17" s="34">
+      <c r="AO17" s="35">
         <v>14000</v>
       </c>
-      <c r="AP17" s="34">
+      <c r="AP17" s="35">
         <v>6800</v>
       </c>
-      <c r="AQ17" s="34">
+      <c r="AQ17" s="35">
         <v>3900</v>
       </c>
-      <c r="AR17" s="34">
+      <c r="AR17" s="35">
         <v>6000</v>
       </c>
     </row>
     <row r="18" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A18" s="37"/>
-      <c r="B18" s="37"/>
-      <c r="C18" s="37"/>
-      <c r="D18" s="37"/>
-      <c r="E18" s="37"/>
-      <c r="F18" s="37"/>
-      <c r="G18" s="37"/>
-      <c r="H18" s="37"/>
-      <c r="I18" s="37"/>
-      <c r="J18" s="37"/>
-      <c r="K18" s="37"/>
-      <c r="L18" s="37"/>
-      <c r="M18" s="37"/>
-      <c r="N18" s="37"/>
-      <c r="O18" s="37"/>
-      <c r="P18" s="37"/>
-      <c r="Q18" s="37"/>
-      <c r="R18" s="37"/>
-      <c r="S18" s="37"/>
-      <c r="T18" s="37"/>
-      <c r="U18" s="37"/>
-      <c r="W18" s="34" t="s">
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
+      <c r="C18" s="42"/>
+      <c r="D18" s="42"/>
+      <c r="E18" s="42"/>
+      <c r="F18" s="42"/>
+      <c r="G18" s="42"/>
+      <c r="H18" s="42"/>
+      <c r="I18" s="42"/>
+      <c r="J18" s="42"/>
+      <c r="K18" s="42"/>
+      <c r="L18" s="42"/>
+      <c r="M18" s="42"/>
+      <c r="N18" s="42"/>
+      <c r="O18" s="42"/>
+      <c r="P18" s="42"/>
+      <c r="Q18" s="42"/>
+      <c r="R18" s="42"/>
+      <c r="S18" s="42"/>
+      <c r="T18" s="42"/>
+      <c r="U18" s="42"/>
+      <c r="W18" s="35" t="s">
         <v>33</v>
       </c>
-      <c r="X18" s="34" t="s">
+      <c r="X18" s="35" t="s">
         <v>33</v>
       </c>
-      <c r="Y18" s="34" t="s">
+      <c r="Y18" s="35" t="s">
         <v>156</v>
       </c>
-      <c r="AA18" s="34" t="s">
+      <c r="AA18" s="35" t="s">
         <v>33</v>
       </c>
-      <c r="AB18" s="34">
+      <c r="AB18" s="35">
         <v>285564</v>
       </c>
-      <c r="AC18" s="34">
+      <c r="AC18" s="35">
         <v>236682</v>
       </c>
-      <c r="AD18" s="34">
+      <c r="AD18" s="35">
         <v>99656</v>
       </c>
-      <c r="AE18" s="34">
+      <c r="AE18" s="35">
         <v>22196</v>
       </c>
-      <c r="AF18" s="34">
+      <c r="AF18" s="35">
         <v>7984</v>
       </c>
-      <c r="AH18" s="34" t="s">
+      <c r="AH18" s="35" t="s">
         <v>33</v>
       </c>
-      <c r="AI18" s="34">
+      <c r="AI18" s="35">
         <v>875000</v>
       </c>
-      <c r="AJ18" s="34">
+      <c r="AJ18" s="35">
         <v>805000</v>
       </c>
-      <c r="AK18" s="34">
+      <c r="AK18" s="35">
         <v>538000</v>
       </c>
-      <c r="AL18" s="34">
+      <c r="AL18" s="35">
         <v>220000</v>
       </c>
-      <c r="AM18" s="34">
+      <c r="AM18" s="35">
         <v>74000</v>
       </c>
-      <c r="AN18" s="34">
+      <c r="AN18" s="35">
         <v>33000</v>
       </c>
-      <c r="AO18" s="34">
+      <c r="AO18" s="35">
         <v>17000</v>
       </c>
-      <c r="AP18" s="34">
+      <c r="AP18" s="35">
         <v>11000</v>
       </c>
-      <c r="AQ18" s="34">
+      <c r="AQ18" s="35">
         <v>8800</v>
       </c>
-      <c r="AR18" s="34">
+      <c r="AR18" s="35">
         <v>23000</v>
       </c>
     </row>
     <row r="19" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A19" s="37"/>
-      <c r="B19" s="37"/>
-      <c r="C19" s="37"/>
-      <c r="D19" s="37"/>
-      <c r="E19" s="37"/>
-      <c r="F19" s="37"/>
-      <c r="G19" s="37"/>
-      <c r="H19" s="37"/>
-      <c r="I19" s="37"/>
-      <c r="J19" s="37"/>
-      <c r="K19" s="37"/>
-      <c r="L19" s="37"/>
-      <c r="M19" s="37"/>
-      <c r="N19" s="37"/>
-      <c r="O19" s="37"/>
-      <c r="P19" s="37"/>
-      <c r="Q19" s="37"/>
-      <c r="R19" s="37"/>
-      <c r="S19" s="37"/>
-      <c r="T19" s="37"/>
-      <c r="U19" s="37"/>
-      <c r="W19" s="34" t="s">
+      <c r="A19" s="42"/>
+      <c r="B19" s="42"/>
+      <c r="C19" s="42"/>
+      <c r="D19" s="42"/>
+      <c r="E19" s="42"/>
+      <c r="F19" s="42"/>
+      <c r="G19" s="42"/>
+      <c r="H19" s="42"/>
+      <c r="I19" s="42"/>
+      <c r="J19" s="42"/>
+      <c r="K19" s="42"/>
+      <c r="L19" s="42"/>
+      <c r="M19" s="42"/>
+      <c r="N19" s="42"/>
+      <c r="O19" s="42"/>
+      <c r="P19" s="42"/>
+      <c r="Q19" s="42"/>
+      <c r="R19" s="42"/>
+      <c r="S19" s="42"/>
+      <c r="T19" s="42"/>
+      <c r="U19" s="42"/>
+      <c r="W19" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="X19" s="34" t="s">
+      <c r="X19" s="35" t="s">
         <v>157</v>
       </c>
-      <c r="Y19" s="34" t="s">
+      <c r="Y19" s="35" t="s">
         <v>158</v>
       </c>
-      <c r="AA19" s="34" t="s">
+      <c r="AA19" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="AB19" s="34">
+      <c r="AB19" s="35">
         <v>190382</v>
       </c>
-      <c r="AC19" s="34">
+      <c r="AC19" s="35">
         <v>214531</v>
       </c>
-      <c r="AD19" s="34">
+      <c r="AD19" s="35">
         <v>94920</v>
       </c>
-      <c r="AE19" s="34">
+      <c r="AE19" s="35">
         <v>17843</v>
       </c>
-      <c r="AF19" s="34">
+      <c r="AF19" s="35">
         <v>4387</v>
       </c>
-      <c r="AH19" s="34" t="s">
+      <c r="AH19" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="AI19" s="34">
+      <c r="AI19" s="35">
         <v>204000</v>
       </c>
-      <c r="AJ19" s="34">
+      <c r="AJ19" s="35">
         <v>197000</v>
       </c>
-      <c r="AK19" s="34">
+      <c r="AK19" s="35">
         <v>226000</v>
       </c>
-      <c r="AL19" s="34">
+      <c r="AL19" s="35">
         <v>137000</v>
       </c>
-      <c r="AM19" s="34">
+      <c r="AM19" s="35">
         <v>60000</v>
       </c>
-      <c r="AN19" s="34">
+      <c r="AN19" s="35">
         <v>26000</v>
       </c>
-      <c r="AO19" s="34">
+      <c r="AO19" s="35">
         <v>12000</v>
       </c>
-      <c r="AP19" s="34">
+      <c r="AP19" s="35">
         <v>7000</v>
       </c>
-      <c r="AQ19" s="34">
+      <c r="AQ19" s="35">
         <v>4600</v>
       </c>
-      <c r="AR19" s="34">
+      <c r="AR19" s="35">
         <v>7600</v>
       </c>
     </row>
     <row r="20" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A20" s="37"/>
-      <c r="B20" s="37"/>
-      <c r="C20" s="37"/>
-      <c r="D20" s="37"/>
-      <c r="E20" s="37"/>
-      <c r="F20" s="37"/>
-      <c r="G20" s="37"/>
-      <c r="H20" s="37"/>
-      <c r="I20" s="37"/>
-      <c r="J20" s="37"/>
-      <c r="K20" s="37"/>
-      <c r="L20" s="37"/>
-      <c r="M20" s="37"/>
-      <c r="N20" s="37"/>
-      <c r="O20" s="37"/>
-      <c r="P20" s="37"/>
-      <c r="Q20" s="37"/>
-      <c r="R20" s="37"/>
-      <c r="S20" s="37"/>
-      <c r="T20" s="37"/>
-      <c r="U20" s="37"/>
-      <c r="W20" s="34" t="s">
+      <c r="A20" s="42"/>
+      <c r="B20" s="42"/>
+      <c r="C20" s="42"/>
+      <c r="D20" s="42"/>
+      <c r="E20" s="42"/>
+      <c r="F20" s="42"/>
+      <c r="G20" s="42"/>
+      <c r="H20" s="42"/>
+      <c r="I20" s="42"/>
+      <c r="J20" s="42"/>
+      <c r="K20" s="42"/>
+      <c r="L20" s="42"/>
+      <c r="M20" s="42"/>
+      <c r="N20" s="42"/>
+      <c r="O20" s="42"/>
+      <c r="P20" s="42"/>
+      <c r="Q20" s="42"/>
+      <c r="R20" s="42"/>
+      <c r="S20" s="42"/>
+      <c r="T20" s="42"/>
+      <c r="U20" s="42"/>
+      <c r="W20" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="Y20" s="34" t="s">
+      <c r="Y20" s="35" t="s">
         <v>159</v>
       </c>
-      <c r="AA20" s="34" t="s">
+      <c r="AA20" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="AB20" s="34">
+      <c r="AB20" s="35">
         <v>0</v>
       </c>
-      <c r="AC20" s="34">
+      <c r="AC20" s="35">
         <v>0</v>
       </c>
-      <c r="AD20" s="34">
+      <c r="AD20" s="35">
         <v>0</v>
       </c>
-      <c r="AE20" s="34">
+      <c r="AE20" s="35">
         <v>0</v>
       </c>
-      <c r="AF20" s="34">
+      <c r="AF20" s="35">
         <v>0</v>
       </c>
-      <c r="AH20" s="34" t="s">
+      <c r="AH20" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="AI20" s="34">
+      <c r="AI20" s="35">
         <v>605000</v>
       </c>
-      <c r="AJ20" s="34">
+      <c r="AJ20" s="35">
         <v>503000</v>
       </c>
-      <c r="AK20" s="34">
+      <c r="AK20" s="35">
         <v>281000</v>
       </c>
-      <c r="AL20" s="34">
+      <c r="AL20" s="35">
         <v>102000</v>
       </c>
-      <c r="AM20" s="34">
+      <c r="AM20" s="35">
         <v>34000</v>
       </c>
-      <c r="AN20" s="34">
+      <c r="AN20" s="35">
         <v>16000</v>
       </c>
-      <c r="AO20" s="34">
+      <c r="AO20" s="35">
         <v>7600</v>
       </c>
-      <c r="AP20" s="34">
+      <c r="AP20" s="35">
         <v>5700</v>
       </c>
-      <c r="AQ20" s="34">
+      <c r="AQ20" s="35">
         <v>5300</v>
       </c>
-      <c r="AR20" s="34">
+      <c r="AR20" s="35">
         <v>24000</v>
       </c>
     </row>
     <row r="21" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A21" s="37"/>
-      <c r="B21" s="37"/>
-      <c r="C21" s="37"/>
-      <c r="D21" s="37"/>
-      <c r="E21" s="37"/>
-      <c r="F21" s="37"/>
-      <c r="G21" s="37"/>
-      <c r="H21" s="37"/>
-      <c r="I21" s="37"/>
-      <c r="J21" s="37"/>
-      <c r="K21" s="37"/>
-      <c r="L21" s="37"/>
-      <c r="M21" s="37"/>
-      <c r="N21" s="37"/>
-      <c r="O21" s="37"/>
-      <c r="P21" s="37"/>
-      <c r="Q21" s="37"/>
-      <c r="R21" s="37"/>
-      <c r="S21" s="37"/>
-      <c r="T21" s="37"/>
-      <c r="U21" s="37"/>
-      <c r="W21" s="34" t="s">
+      <c r="A21" s="42"/>
+      <c r="B21" s="42"/>
+      <c r="C21" s="42"/>
+      <c r="D21" s="42"/>
+      <c r="E21" s="42"/>
+      <c r="F21" s="42"/>
+      <c r="G21" s="42"/>
+      <c r="H21" s="42"/>
+      <c r="I21" s="42"/>
+      <c r="J21" s="42"/>
+      <c r="K21" s="42"/>
+      <c r="L21" s="42"/>
+      <c r="M21" s="42"/>
+      <c r="N21" s="42"/>
+      <c r="O21" s="42"/>
+      <c r="P21" s="42"/>
+      <c r="Q21" s="42"/>
+      <c r="R21" s="42"/>
+      <c r="S21" s="42"/>
+      <c r="T21" s="42"/>
+      <c r="U21" s="42"/>
+      <c r="W21" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="X21" s="34" t="s">
+      <c r="X21" s="35" t="s">
         <v>53</v>
       </c>
-      <c r="Y21" s="34" t="s">
+      <c r="Y21" s="35" t="s">
         <v>160</v>
       </c>
-      <c r="AA21" s="34" t="s">
+      <c r="AA21" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="AB21" s="34">
+      <c r="AB21" s="35">
         <v>1087503</v>
       </c>
-      <c r="AC21" s="34">
+      <c r="AC21" s="35">
         <v>879291</v>
       </c>
-      <c r="AD21" s="34">
+      <c r="AD21" s="35">
         <v>371115</v>
       </c>
-      <c r="AE21" s="34">
+      <c r="AE21" s="35">
         <v>98132</v>
       </c>
-      <c r="AF21" s="34">
+      <c r="AF21" s="35">
         <v>45854</v>
       </c>
-      <c r="AH21" s="34" t="s">
+      <c r="AH21" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="AI21" s="34">
+      <c r="AI21" s="35">
         <v>87000</v>
       </c>
-      <c r="AJ21" s="34">
+      <c r="AJ21" s="35">
         <v>80000</v>
       </c>
-      <c r="AK21" s="34">
+      <c r="AK21" s="35">
         <v>66000</v>
       </c>
-      <c r="AL21" s="34">
+      <c r="AL21" s="35">
         <v>30000</v>
       </c>
-      <c r="AM21" s="34">
+      <c r="AM21" s="35">
         <v>12000</v>
       </c>
-      <c r="AN21" s="34">
+      <c r="AN21" s="35">
         <v>6100</v>
       </c>
-      <c r="AO21" s="34">
+      <c r="AO21" s="35">
         <v>3400</v>
       </c>
-      <c r="AP21" s="34">
+      <c r="AP21" s="35">
         <v>2400</v>
       </c>
-      <c r="AQ21" s="34">
+      <c r="AQ21" s="35">
         <v>2100</v>
       </c>
-      <c r="AR21" s="34">
+      <c r="AR21" s="35">
         <v>7300</v>
       </c>
     </row>
     <row r="22" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A22" s="37"/>
-      <c r="B22" s="37"/>
-      <c r="C22" s="37"/>
-      <c r="D22" s="37"/>
-      <c r="E22" s="37"/>
-      <c r="F22" s="37"/>
-      <c r="G22" s="37"/>
-      <c r="H22" s="37"/>
-      <c r="I22" s="37"/>
-      <c r="J22" s="37"/>
-      <c r="K22" s="37"/>
-      <c r="L22" s="37"/>
-      <c r="M22" s="37"/>
-      <c r="N22" s="37"/>
-      <c r="O22" s="37"/>
-      <c r="P22" s="37"/>
-      <c r="Q22" s="37"/>
-      <c r="R22" s="37"/>
-      <c r="S22" s="37"/>
-      <c r="T22" s="37"/>
-      <c r="U22" s="37"/>
+      <c r="A22" s="42"/>
+      <c r="B22" s="42"/>
+      <c r="C22" s="42"/>
+      <c r="D22" s="42"/>
+      <c r="E22" s="42"/>
+      <c r="F22" s="42"/>
+      <c r="G22" s="42"/>
+      <c r="H22" s="42"/>
+      <c r="I22" s="42"/>
+      <c r="J22" s="42"/>
+      <c r="K22" s="42"/>
+      <c r="L22" s="42"/>
+      <c r="M22" s="42"/>
+      <c r="N22" s="42"/>
+      <c r="O22" s="42"/>
+      <c r="P22" s="42"/>
+      <c r="Q22" s="42"/>
+      <c r="R22" s="42"/>
+      <c r="S22" s="42"/>
+      <c r="T22" s="42"/>
+      <c r="U22" s="42"/>
     </row>
     <row r="23" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A23" s="37"/>
-      <c r="B23" s="37"/>
-      <c r="C23" s="37"/>
-      <c r="D23" s="37"/>
-      <c r="E23" s="37"/>
-      <c r="F23" s="37"/>
-      <c r="G23" s="37"/>
-      <c r="H23" s="37"/>
-      <c r="I23" s="37"/>
-      <c r="J23" s="37"/>
-      <c r="K23" s="37"/>
-      <c r="L23" s="37"/>
-      <c r="M23" s="37"/>
-      <c r="N23" s="37"/>
-      <c r="O23" s="37"/>
-      <c r="P23" s="37"/>
-      <c r="Q23" s="37"/>
-      <c r="R23" s="37"/>
-      <c r="S23" s="37"/>
-      <c r="T23" s="37"/>
-      <c r="U23" s="37"/>
+      <c r="A23" s="42"/>
+      <c r="B23" s="42"/>
+      <c r="C23" s="42"/>
+      <c r="D23" s="42"/>
+      <c r="E23" s="42"/>
+      <c r="F23" s="42"/>
+      <c r="G23" s="42"/>
+      <c r="H23" s="42"/>
+      <c r="I23" s="42"/>
+      <c r="J23" s="42"/>
+      <c r="K23" s="42"/>
+      <c r="L23" s="42"/>
+      <c r="M23" s="42"/>
+      <c r="N23" s="42"/>
+      <c r="O23" s="42"/>
+      <c r="P23" s="42"/>
+      <c r="Q23" s="42"/>
+      <c r="R23" s="42"/>
+      <c r="S23" s="42"/>
+      <c r="T23" s="42"/>
+      <c r="U23" s="42"/>
     </row>
     <row r="24" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A24" s="37"/>
-      <c r="B24" s="37"/>
-      <c r="C24" s="37"/>
-      <c r="D24" s="37"/>
-      <c r="E24" s="37"/>
-      <c r="F24" s="37"/>
-      <c r="G24" s="37"/>
-      <c r="H24" s="37"/>
-      <c r="I24" s="37"/>
-      <c r="J24" s="37"/>
-      <c r="K24" s="37"/>
-      <c r="L24" s="37"/>
-      <c r="M24" s="37"/>
-      <c r="N24" s="37"/>
-      <c r="O24" s="37"/>
-      <c r="P24" s="37"/>
-      <c r="Q24" s="37"/>
-      <c r="R24" s="37"/>
-      <c r="S24" s="37"/>
-      <c r="T24" s="37"/>
-      <c r="U24" s="37"/>
+      <c r="A24" s="42"/>
+      <c r="B24" s="42"/>
+      <c r="C24" s="42"/>
+      <c r="D24" s="42"/>
+      <c r="E24" s="42"/>
+      <c r="F24" s="42"/>
+      <c r="G24" s="42"/>
+      <c r="H24" s="42"/>
+      <c r="I24" s="42"/>
+      <c r="J24" s="42"/>
+      <c r="K24" s="42"/>
+      <c r="L24" s="42"/>
+      <c r="M24" s="42"/>
+      <c r="N24" s="42"/>
+      <c r="O24" s="42"/>
+      <c r="P24" s="42"/>
+      <c r="Q24" s="42"/>
+      <c r="R24" s="42"/>
+      <c r="S24" s="42"/>
+      <c r="T24" s="42"/>
+      <c r="U24" s="42"/>
     </row>
     <row r="25" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A25" s="37"/>
-      <c r="B25" s="37"/>
-      <c r="C25" s="37"/>
-      <c r="D25" s="37"/>
-      <c r="E25" s="37"/>
-      <c r="F25" s="37"/>
-      <c r="G25" s="37"/>
-      <c r="H25" s="37"/>
-      <c r="I25" s="37"/>
-      <c r="J25" s="37"/>
-      <c r="K25" s="37"/>
-      <c r="L25" s="37"/>
-      <c r="M25" s="37"/>
-      <c r="N25" s="37"/>
-      <c r="O25" s="37"/>
-      <c r="P25" s="37"/>
-      <c r="Q25" s="37"/>
-      <c r="R25" s="37"/>
-      <c r="S25" s="37"/>
-      <c r="T25" s="37"/>
-      <c r="U25" s="37"/>
+      <c r="A25" s="42"/>
+      <c r="B25" s="42"/>
+      <c r="C25" s="42"/>
+      <c r="D25" s="42"/>
+      <c r="E25" s="42"/>
+      <c r="F25" s="42"/>
+      <c r="G25" s="42"/>
+      <c r="H25" s="42"/>
+      <c r="I25" s="42"/>
+      <c r="J25" s="42"/>
+      <c r="K25" s="42"/>
+      <c r="L25" s="42"/>
+      <c r="M25" s="42"/>
+      <c r="N25" s="42"/>
+      <c r="O25" s="42"/>
+      <c r="P25" s="42"/>
+      <c r="Q25" s="42"/>
+      <c r="R25" s="42"/>
+      <c r="S25" s="42"/>
+      <c r="T25" s="42"/>
+      <c r="U25" s="42"/>
     </row>
     <row r="26" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A26" s="37"/>
-      <c r="B26" s="37"/>
-      <c r="C26" s="37"/>
-      <c r="D26" s="37"/>
-      <c r="E26" s="37"/>
-      <c r="F26" s="37"/>
-      <c r="G26" s="37"/>
-      <c r="H26" s="37"/>
-      <c r="I26" s="37"/>
-      <c r="J26" s="37"/>
-      <c r="K26" s="37"/>
-      <c r="L26" s="37"/>
-      <c r="M26" s="37"/>
-      <c r="N26" s="37"/>
-      <c r="O26" s="37"/>
-      <c r="P26" s="37"/>
-      <c r="Q26" s="37"/>
-      <c r="R26" s="37"/>
-      <c r="S26" s="37"/>
-      <c r="T26" s="37"/>
-      <c r="U26" s="37"/>
+      <c r="A26" s="42"/>
+      <c r="B26" s="42"/>
+      <c r="C26" s="42"/>
+      <c r="D26" s="42"/>
+      <c r="E26" s="42"/>
+      <c r="F26" s="42"/>
+      <c r="G26" s="42"/>
+      <c r="H26" s="42"/>
+      <c r="I26" s="42"/>
+      <c r="J26" s="42"/>
+      <c r="K26" s="42"/>
+      <c r="L26" s="42"/>
+      <c r="M26" s="42"/>
+      <c r="N26" s="42"/>
+      <c r="O26" s="42"/>
+      <c r="P26" s="42"/>
+      <c r="Q26" s="42"/>
+      <c r="R26" s="42"/>
+      <c r="S26" s="42"/>
+      <c r="T26" s="42"/>
+      <c r="U26" s="42"/>
     </row>
     <row r="27" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A27" s="37"/>
-      <c r="B27" s="37"/>
-      <c r="C27" s="37"/>
-      <c r="D27" s="37"/>
-      <c r="E27" s="37"/>
-      <c r="F27" s="37"/>
-      <c r="G27" s="37"/>
-      <c r="H27" s="37"/>
-      <c r="I27" s="37"/>
-      <c r="J27" s="37"/>
-      <c r="K27" s="37"/>
-      <c r="L27" s="37"/>
-      <c r="M27" s="37"/>
-      <c r="N27" s="37"/>
-      <c r="O27" s="37"/>
-      <c r="P27" s="37"/>
-      <c r="Q27" s="37"/>
-      <c r="R27" s="37"/>
-      <c r="S27" s="37"/>
-      <c r="T27" s="37"/>
-      <c r="U27" s="37"/>
+      <c r="A27" s="42"/>
+      <c r="B27" s="42"/>
+      <c r="C27" s="42"/>
+      <c r="D27" s="42"/>
+      <c r="E27" s="42"/>
+      <c r="F27" s="42"/>
+      <c r="G27" s="42"/>
+      <c r="H27" s="42"/>
+      <c r="I27" s="42"/>
+      <c r="J27" s="42"/>
+      <c r="K27" s="42"/>
+      <c r="L27" s="42"/>
+      <c r="M27" s="42"/>
+      <c r="N27" s="42"/>
+      <c r="O27" s="42"/>
+      <c r="P27" s="42"/>
+      <c r="Q27" s="42"/>
+      <c r="R27" s="42"/>
+      <c r="S27" s="42"/>
+      <c r="T27" s="42"/>
+      <c r="U27" s="42"/>
     </row>
     <row r="28" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A28" s="37"/>
-      <c r="B28" s="37"/>
-      <c r="C28" s="37"/>
-      <c r="D28" s="37"/>
-      <c r="E28" s="37"/>
-      <c r="F28" s="37"/>
-      <c r="G28" s="37"/>
-      <c r="H28" s="37"/>
-      <c r="I28" s="37"/>
-      <c r="J28" s="37"/>
-      <c r="K28" s="37"/>
-      <c r="L28" s="37"/>
-      <c r="M28" s="37"/>
-      <c r="N28" s="37"/>
-      <c r="O28" s="37"/>
-      <c r="P28" s="37"/>
-      <c r="Q28" s="37"/>
-      <c r="R28" s="37"/>
-      <c r="S28" s="37"/>
-      <c r="T28" s="37"/>
-      <c r="U28" s="37"/>
+      <c r="A28" s="42"/>
+      <c r="B28" s="42"/>
+      <c r="C28" s="42"/>
+      <c r="D28" s="42"/>
+      <c r="E28" s="42"/>
+      <c r="F28" s="42"/>
+      <c r="G28" s="42"/>
+      <c r="H28" s="42"/>
+      <c r="I28" s="42"/>
+      <c r="J28" s="42"/>
+      <c r="K28" s="42"/>
+      <c r="L28" s="42"/>
+      <c r="M28" s="42"/>
+      <c r="N28" s="42"/>
+      <c r="O28" s="42"/>
+      <c r="P28" s="42"/>
+      <c r="Q28" s="42"/>
+      <c r="R28" s="42"/>
+      <c r="S28" s="42"/>
+      <c r="T28" s="42"/>
+      <c r="U28" s="42"/>
     </row>
     <row r="29" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A29" s="37"/>
-      <c r="B29" s="37"/>
-      <c r="C29" s="37"/>
-      <c r="D29" s="37"/>
-      <c r="E29" s="37"/>
-      <c r="F29" s="37"/>
-      <c r="G29" s="37"/>
-      <c r="H29" s="37"/>
-      <c r="I29" s="37"/>
-      <c r="J29" s="37"/>
-      <c r="K29" s="37"/>
-      <c r="L29" s="37"/>
-      <c r="M29" s="37"/>
-      <c r="N29" s="37"/>
-      <c r="O29" s="37"/>
-      <c r="P29" s="37"/>
-      <c r="Q29" s="37"/>
-      <c r="R29" s="37"/>
-      <c r="S29" s="37"/>
-      <c r="T29" s="37"/>
-      <c r="U29" s="37"/>
+      <c r="A29" s="42"/>
+      <c r="B29" s="42"/>
+      <c r="C29" s="42"/>
+      <c r="D29" s="42"/>
+      <c r="E29" s="42"/>
+      <c r="F29" s="42"/>
+      <c r="G29" s="42"/>
+      <c r="H29" s="42"/>
+      <c r="I29" s="42"/>
+      <c r="J29" s="42"/>
+      <c r="K29" s="42"/>
+      <c r="L29" s="42"/>
+      <c r="M29" s="42"/>
+      <c r="N29" s="42"/>
+      <c r="O29" s="42"/>
+      <c r="P29" s="42"/>
+      <c r="Q29" s="42"/>
+      <c r="R29" s="42"/>
+      <c r="S29" s="42"/>
+      <c r="T29" s="42"/>
+      <c r="U29" s="42"/>
     </row>
     <row r="30" spans="1:44" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="37" t="s">
+      <c r="A30" s="42" t="s">
         <v>171</v>
       </c>
-      <c r="B30" s="37" t="s">
+      <c r="B30" s="42" t="s">
         <v>172</v>
       </c>
-      <c r="C30" s="37"/>
-      <c r="D30" s="37" t="s">
+      <c r="C30" s="42"/>
+      <c r="D30" s="42" t="s">
         <v>173</v>
       </c>
-      <c r="E30" s="37" t="s">
+      <c r="E30" s="42" t="s">
         <v>174</v>
       </c>
-      <c r="F30" s="37"/>
-      <c r="G30" s="37"/>
-      <c r="H30" s="37"/>
-      <c r="I30" s="37"/>
-      <c r="J30" s="37"/>
-      <c r="K30" s="37"/>
-      <c r="L30" s="37"/>
-      <c r="M30" s="37"/>
-      <c r="N30" s="37"/>
-      <c r="O30" s="37"/>
-      <c r="P30" s="37"/>
-      <c r="Q30" s="37"/>
-      <c r="R30" s="37"/>
-      <c r="S30" s="37"/>
-      <c r="T30" s="37"/>
-      <c r="U30" s="37"/>
+      <c r="F30" s="42"/>
+      <c r="G30" s="42"/>
+      <c r="H30" s="42"/>
+      <c r="I30" s="42"/>
+      <c r="J30" s="42"/>
+      <c r="K30" s="42"/>
+      <c r="L30" s="42"/>
+      <c r="M30" s="42"/>
+      <c r="N30" s="42"/>
+      <c r="O30" s="42"/>
+      <c r="P30" s="42"/>
+      <c r="Q30" s="42"/>
+      <c r="R30" s="42"/>
+      <c r="S30" s="42"/>
+      <c r="T30" s="42"/>
+      <c r="U30" s="42"/>
     </row>
     <row r="31" spans="1:44" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="34" t="s">
+      <c r="A31" s="35" t="s">
         <v>47</v>
       </c>
-      <c r="B31" s="34">
+      <c r="B31" s="35">
         <f>INDEX($AA$2:$AF$21,MATCH($I$4,$AA$2:$AA$21,0),6)</f>
         <v>5601</v>
       </c>
-      <c r="D31" s="34" t="s">
+      <c r="D31" s="35" t="s">
         <v>100</v>
       </c>
-      <c r="E31" s="34">
+      <c r="E31" s="35">
         <f>INDEX($AH$2:$AR$21,MATCH($I$4,$AH$2:$AH$21,0),2)</f>
         <v>1100000</v>
       </c>
     </row>
     <row r="32" spans="1:44" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="34" t="s">
+      <c r="A32" s="35" t="s">
         <v>48</v>
       </c>
-      <c r="B32" s="34">
+      <c r="B32" s="35">
         <f>INDEX($AA$2:$AF$21,MATCH($I$4,$AA$2:$AA$21,0),5)</f>
         <v>10170</v>
       </c>
-      <c r="D32" s="34" t="s">
+      <c r="D32" s="35" t="s">
         <v>99</v>
       </c>
-      <c r="E32" s="34">
+      <c r="E32" s="35">
         <f>INDEX($AH$2:$AR$21,MATCH($I$4,$AH$2:$AH$21,0),3)</f>
         <v>557000</v>
       </c>
     </row>
     <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="34" t="s">
+      <c r="A33" s="35" t="s">
         <v>49</v>
       </c>
-      <c r="B33" s="34">
+      <c r="B33" s="35">
         <f>INDEX($AA$2:$AF$21,MATCH($I$4,$AA$2:$AA$21,0),4)</f>
         <v>46266</v>
       </c>
-      <c r="D33" s="34" t="s">
+      <c r="D33" s="35" t="s">
         <v>98</v>
       </c>
-      <c r="E33" s="34">
+      <c r="E33" s="35">
         <f>INDEX($AH$2:$AR$21,MATCH($I$4,$AH$2:$AH$21,0),4)</f>
         <v>280000</v>
       </c>
     </row>
     <row r="34" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="34" t="s">
+      <c r="A34" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="B34" s="34">
+      <c r="B34" s="35">
         <f>INDEX($AA$2:$AF$21,MATCH($I$4,$AA$2:$AA$21,0),3)</f>
         <v>137019</v>
       </c>
-      <c r="D34" s="34" t="s">
+      <c r="D34" s="35" t="s">
         <v>97</v>
       </c>
-      <c r="E34" s="34">
+      <c r="E34" s="35">
         <f>INDEX($AH$2:$AR$21,MATCH($I$4,$AH$2:$AH$21,0),5)</f>
         <v>110000</v>
       </c>
     </row>
     <row r="35" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="34" t="s">
+      <c r="A35" s="35" t="s">
         <v>51</v>
       </c>
-      <c r="B35" s="34">
+      <c r="B35" s="35">
         <f>INDEX($AA$2:$AF$21,MATCH($I$4,$AA$2:$AA$21,0),2)</f>
         <v>271164</v>
       </c>
-      <c r="D35" s="34" t="s">
+      <c r="D35" s="35" t="s">
         <v>96</v>
       </c>
-      <c r="E35" s="34">
+      <c r="E35" s="35">
         <f>INDEX($AH$2:$AR$21,MATCH($I$4,$AH$2:$AH$21,0),6)</f>
         <v>41000</v>
       </c>
     </row>
     <row r="36" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
-      <c r="D36" s="34" t="s">
+      <c r="D36" s="35" t="s">
         <v>47</v>
       </c>
-      <c r="E36" s="34">
+      <c r="E36" s="35">
         <f>INDEX($AH$2:$AR$21,MATCH($I$4,$AH$2:$AH$21,0),7)</f>
         <v>22000</v>
       </c>
     </row>
     <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
-      <c r="D37" s="34" t="s">
+      <c r="D37" s="35" t="s">
         <v>48</v>
       </c>
-      <c r="E37" s="34">
+      <c r="E37" s="35">
         <f>INDEX($AH$2:$AR$21,MATCH($I$4,$AH$2:$AH$21,0),8)</f>
         <v>11000</v>
       </c>
     </row>
     <row r="38" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
-      <c r="D38" s="34" t="s">
+      <c r="D38" s="35" t="s">
         <v>49</v>
       </c>
-      <c r="E38" s="34">
+      <c r="E38" s="35">
         <f>INDEX($AH$2:$AR$21,MATCH($I$4,$AH$2:$AH$21,0),9)</f>
         <v>8400</v>
       </c>
     </row>
     <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
-      <c r="D39" s="34" t="s">
+      <c r="D39" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="E39" s="34">
+      <c r="E39" s="35">
         <f>INDEX($AH$2:$AR$21,MATCH($I$4,$AH$2:$AH$21,0),10)</f>
         <v>7500</v>
       </c>
     </row>
     <row r="40" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
-      <c r="D40" s="34" t="s">
+      <c r="D40" s="35" t="s">
         <v>51</v>
       </c>
-      <c r="E40" s="34">
+      <c r="E40" s="35">
         <f>INDEX($AH$2:$AR$21,MATCH($I$4,$AH$2:$AH$21,0),11)</f>
         <v>44000</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="17">
-    <mergeCell ref="A1:U1"/>
-    <mergeCell ref="I4:M4"/>
-    <mergeCell ref="I3:M3"/>
-    <mergeCell ref="N7:U7"/>
-    <mergeCell ref="A7:H7"/>
     <mergeCell ref="O14:U14"/>
     <mergeCell ref="B9:H9"/>
     <mergeCell ref="B10:H10"/>
@@ -51211,6 +51205,11 @@
     <mergeCell ref="O11:U11"/>
     <mergeCell ref="O12:U12"/>
     <mergeCell ref="O13:U13"/>
+    <mergeCell ref="A1:U1"/>
+    <mergeCell ref="I4:M4"/>
+    <mergeCell ref="I3:M3"/>
+    <mergeCell ref="N7:U7"/>
+    <mergeCell ref="A7:H7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>